<commit_message>
Enrich B-category premium indicators: add liability, accident, commercial property, guarantee, cargo transportation premiums
</commit_message>
<xml_diff>
--- a/agents/zd-agent0811/indicator/indicator_dictionary.xlsx
+++ b/agents/zd-agent0811/indicator/indicator_dictionary.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1868,6 +1868,266 @@
       <c r="J25" s="25" t="inlineStr">
         <is>
           <t>偿付能力信息|风险管理|监管指标</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>B013</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>业务规模指标</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>责任保险保费</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>责任险保费|责任保险保费收入|责任险保费收入|liability insurance premium</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>责任保险保费收入|责任险保费收入|责任保险原保险保费收入|责任险原保险保费收入|责任保险业务保费收入|责任险业务保费收入|责任保险保费|责任险保费|责任保险|责任险|其他责任保险|责任保险业务|liability insurance premium|責任保險保費收入|責任險保費收入</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>责任保险业务保费收入。</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>百万元</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>按责任保险业务披露的保费金额提取；如披露单位为亿元，统一换算为百万元；不得提取同比增长率或变化百分点。</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>经营情况分析|业务结构|分部信息|保费收入公告</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>B014</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>业务规模指标</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>意外伤害保险保费</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>意外险保费|意外伤害险保费|accident insurance premium</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>意外伤害保险保费收入|意外险保费收入|意外伤害险保费收入|意外伤害保险原保险保费收入|意外险原保险保费收入|意外伤害保险业务保费收入|意外险业务保费收入|意外伤害保险保费|意外险保费|意外伤害保险|意外险|意外伤害险|意外险业务|accident insurance premium|意外傷害保險保費收入|意外險保費收入</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>意外伤害保险业务保费收入。</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>百万元</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>按意外伤害保险业务披露的保费金额提取；如披露单位为亿元，统一换算为百万元；不得提取同比增长率或变化百分点。</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>经营情况分析|业务结构|分部信息|保费收入公告</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>B015</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>业务规模指标</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>企财险保费</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>企业财产保险保费|企业财产险保费|commercial property insurance premium</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>企财险保费收入|企业财产保险保费收入|企业财产险保费收入|企财险原保险保费收入|企业财产保险原保险保费收入|企财险业务保费收入|企业财产保险业务保费收入|企财险保费|企业财产保险保费|企财险|企业财产保险|企业财产险|企财险业务|commercial property insurance premium|企業財產保險保費收入|企財險保費收入</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>企业财产保险业务保费收入。</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>百万元</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>按企业财产保险业务披露的保费金额提取；如披露单位为亿元，统一换算为百万元；不得提取同比增长率或变化百分点。</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>经营情况分析|业务结构|分部信息|保费收入公告</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>B016</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>业务规模指标</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>保证保险保费</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>保证险保费|guarantee insurance premium</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>保证保险保费收入|保证险保费收入|保证保险原保险保费收入|保证险原保险保费收入|保证保险业务保费收入|保证险业务保费收入|保证保险保费|保证险保费|保证保险|保证险|保证保险业务|guarantee insurance premium|保證保險保費收入|保證險保費收入</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>保证保险业务保费收入。</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>百万元</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>按保证保险业务披露的保费金额提取；如披露单位为亿元，统一换算为百万元；不得提取同比增长率或变化百分点。</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>经营情况分析|业务结构|分部信息|保费收入公告</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>B017</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>业务规模指标</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>货物运输保险保费</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>货运险保费|货物运输险保费|cargo transportation insurance premium</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>货物运输保险保费收入|货运险保费收入|货物运输险保费收入|货物运输保险原保险保费收入|货运险原保险保费收入|货物运输保险业务保费收入|货运险业务保费收入|货物运输保险保费|货运险保费|货物运输保险|货运险|货物运输险|货运险业务|cargo transportation insurance premium|貨物運輸保險保費收入|貨運險保費收入</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>货物运输保险业务保费收入。</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>百万元</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>按货物运输保险业务披露的保费金额提取；如披露单位为亿元，统一换算为百万元；不得提取同比增长率或变化百分点。</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>经营情况分析|业务结构|分部信息|保费收入公告</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove confidence column from extraction results; expand keywords for new B-class premium indicators (traditional Chinese variants)
</commit_message>
<xml_diff>
--- a/agents/zd-agent0811/indicator/indicator_dictionary.xlsx
+++ b/agents/zd-agent0811/indicator/indicator_dictionary.xlsx
@@ -1894,7 +1894,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>责任保险保费收入|责任险保费收入|责任保险原保险保费收入|责任险原保险保费收入|责任保险业务保费收入|责任险业务保费收入|责任保险保费|责任险保费|责任保险|责任险|其他责任保险|责任保险业务|liability insurance premium|責任保險保費收入|責任險保費收入</t>
+          <t>责任保险保费收入|责任险保费收入|责任保险原保险保费收入|责任险原保险保费收入|责任保险业务保费收入|责任险业务保费收入|责任保险保费|责任险保费|责任保险|责任险|其他责任保险|责任保险业务|liability insurance premium|責任保險保費收入|責任險保費收入|責任保險|責任險|責任保險保費|責任險保費|責任保險業務|liability insurance</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>意外伤害保险保费收入|意外险保费收入|意外伤害险保费收入|意外伤害保险原保险保费收入|意外险原保险保费收入|意外伤害保险业务保费收入|意外险业务保费收入|意外伤害保险保费|意外险保费|意外伤害保险|意外险|意外伤害险|意外险业务|accident insurance premium|意外傷害保險保費收入|意外險保費收入</t>
+          <t>意外伤害保险保费收入|意外险保费收入|意外伤害险保费收入|意外伤害保险原保险保费收入|意外险原保险保费收入|意外伤害保险业务保费收入|意外险业务保费收入|意外伤害保险保费|意外险保费|意外伤害保险|意外险|意外伤害险|意外险业务|accident insurance premium|意外傷害保險保費收入|意外險保費收入|意外伤害|意外傷害|意外伤害保险业务|意外傷害保險業務|意外伤害及健康保险|意外傷害及健康險|意外健康险|意外健康險</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>企财险保费收入|企业财产保险保费收入|企业财产险保费收入|企财险原保险保费收入|企业财产保险原保险保费收入|企财险业务保费收入|企业财产保险业务保费收入|企财险保费|企业财产保险保费|企财险|企业财产保险|企业财产险|企财险业务|commercial property insurance premium|企業財產保險保費收入|企財險保費收入</t>
+          <t>企财险保费收入|企业财产保险保费收入|企业财产险保费收入|企财险原保险保费收入|企业财产保险原保险保费收入|企财险业务保费收入|企业财产保险业务保费收入|企财险保费|企业财产保险保费|企财险|企业财产保险|企业财产险|企财险业务|commercial property insurance premium|企業財產保險保費收入|企財險保費收入|企業財產保險|企業財產險|企業財產保險保費|企財險|企財險保費</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>保证保险保费收入|保证险保费收入|保证保险原保险保费收入|保证险原保险保费收入|保证保险业务保费收入|保证险业务保费收入|保证保险保费|保证险保费|保证保险|保证险|保证保险业务|guarantee insurance premium|保證保險保費收入|保證險保費收入</t>
+          <t>保证保险保费收入|保证险保费收入|保证保险原保险保费收入|保证险原保险保费收入|保证保险业务保费收入|保证险业务保费收入|保证保险保费|保证险保费|保证保险|保证险|保证保险业务|guarantee insurance premium|保證保險保費收入|保證險保費收入|保證保險|保證險|保證保險保費|保證險保費</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>货物运输保险保费收入|货运险保费收入|货物运输险保费收入|货物运输保险原保险保费收入|货运险原保险保费收入|货物运输保险业务保费收入|货运险业务保费收入|货物运输保险保费|货运险保费|货物运输保险|货运险|货物运输险|货运险业务|cargo transportation insurance premium|貨物運輸保險保費收入|貨運險保費收入</t>
+          <t>货物运输保险保费收入|货运险保费收入|货物运输险保费收入|货物运输保险原保险保费收入|货运险原保险保费收入|货物运输保险业务保费收入|货运险业务保费收入|货物运输保险保费|货运险保费|货物运输保险|货运险|货物运输险|货运险业务|cargo transportation insurance premium|貨物運輸保險保費收入|貨運險保費收入|貨物運輸保險|貨運險|貨物運輸險|貨物運輸保險保費|貨運險保費</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">

</xml_diff>

<commit_message>
feat: business_scope 口径标准化，新增 business_scope_type 字段与审核功能
保留原始 business_scope，新增标准化字段 business_scope_type；审核页面增加标准业务口径下拉，分析接口支持按口径筛选，并同步指标字典与数据库。
</commit_message>
<xml_diff>
--- a/agents/zd-agent0811/indicator/indicator_dictionary.xlsx
+++ b/agents/zd-agent0811/indicator/indicator_dictionary.xlsx
@@ -4017,7 +4017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4212,6 +4212,40 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>business_scope</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>原始业务范围，保留 LLM 提取或人工修改后的原始描述。</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>太保产险单体（不含太平洋安信农险）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>business_scope_type</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>标准化口径分类，枚举：集团口径 / 财险口径 / 特殊财险口径；由业务口径标准化层生成，可在人工审核页面修正。</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>特殊财险口径</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>